<commit_message>
upsolved all leetcode contest questions of today!
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="91">
   <si>
     <t>date</t>
   </si>
@@ -265,6 +265,30 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/surrounded-regions/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contest Qn: Find Smallest Balanced Index</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/contest/weekly-contest-492/problems/find-the-smallest-balanced-index/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min Capacity Box</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-capacity-box/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min. opns. to sort a string</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-operations-to-sort-a-string/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min cost to partition a binary string</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/contest/weekly-contest-492/problems/minimum-cost-to-partition-a-binary-string/</t>
   </si>
 </sst>
 </file>
@@ -305,14 +329,13 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -814,7 +837,7 @@
   <cols>
     <col bestFit="1" min="1" max="1" width="12.30078125"/>
     <col bestFit="1" min="2" max="2" width="35.98046875"/>
-    <col bestFit="1" min="3" max="3" width="79.98046875"/>
+    <col bestFit="1" min="3" max="3" width="96.87109375"/>
     <col bestFit="1" min="4" max="4" width="21.69140625"/>
   </cols>
   <sheetData>
@@ -1256,7 +1279,7 @@
       </c>
     </row>
     <row r="41" ht="14.25">
-      <c r="A41" s="4">
+      <c r="A41" s="1">
         <v>46088</v>
       </c>
       <c r="B41" t="s">
@@ -1264,6 +1287,44 @@
       </c>
       <c r="C41" s="2" t="s">
         <v>82</v>
+      </c>
+    </row>
+    <row r="42" ht="14.25">
+      <c r="A42" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B42" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="A43" s="1">
+        <v>46089</v>
+      </c>
+      <c r="B43" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="44" ht="14.25">
+      <c r="B44" t="s">
+        <v>87</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="B45" t="s">
+        <v>89</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1307,6 +1368,10 @@
     <hyperlink r:id="rId37" ref="C39"/>
     <hyperlink r:id="rId38" ref="C40"/>
     <hyperlink r:id="rId39" ref="C41"/>
+    <hyperlink r:id="rId40" ref="C42"/>
+    <hyperlink r:id="rId41" ref="C43"/>
+    <hyperlink r:id="rId42" ref="C44"/>
+    <hyperlink r:id="rId43" ref="C45"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem : evaluate division
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>date</t>
   </si>
@@ -295,6 +295,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/clone-graph/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">evaluate division</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/evaluate-division/</t>
   </si>
 </sst>
 </file>
@@ -1319,7 +1325,7 @@
       </c>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="4">
+      <c r="A44" s="1">
         <v>46089</v>
       </c>
       <c r="B44" t="s">
@@ -1330,7 +1336,7 @@
       </c>
     </row>
     <row r="45" ht="14.25">
-      <c r="A45" s="4">
+      <c r="A45" s="1">
         <v>46089</v>
       </c>
       <c r="B45" t="s">
@@ -1341,7 +1347,7 @@
       </c>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="4">
+      <c r="A46" s="1">
         <v>46089</v>
       </c>
       <c r="B46" t="s">
@@ -1349,6 +1355,17 @@
       </c>
       <c r="C46" s="2" t="s">
         <v>92</v>
+      </c>
+    </row>
+    <row r="47" ht="14.25">
+      <c r="A47" s="4">
+        <v>46090</v>
+      </c>
+      <c r="B47" t="s">
+        <v>93</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1397,6 +1414,7 @@
     <hyperlink r:id="rId42" ref="C44"/>
     <hyperlink r:id="rId43" ref="C45"/>
     <hyperlink r:id="rId44" ref="C46"/>
+    <hyperlink r:id="rId45" ref="C47"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
problem: Snakes and Ladders
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>date</t>
   </si>
@@ -331,6 +331,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/course-schedule-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Snakes and Ladders</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/snakes-and-ladders/</t>
   </si>
 </sst>
 </file>
@@ -1452,6 +1458,14 @@
         <v>104</v>
       </c>
     </row>
+    <row r="53" ht="14.25">
+      <c r="B53" t="s">
+        <v>105</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -1504,6 +1518,7 @@
     <hyperlink r:id="rId48" ref="C50"/>
     <hyperlink r:id="rId49" ref="C51"/>
     <hyperlink r:id="rId50" ref="C52"/>
+    <hyperlink r:id="rId51" ref="C53"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Max Depth of Binary Tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>date</t>
   </si>
@@ -409,6 +409,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/largest-rectangle-in-histogram/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max depth of binary tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/maximum-depth-of-binary-tree/</t>
   </si>
 </sst>
 </file>
@@ -1653,7 +1659,7 @@
       </c>
     </row>
     <row r="64" ht="14.25">
-      <c r="A64" s="4">
+      <c r="A64" s="1">
         <v>46100</v>
       </c>
       <c r="B64" t="s">
@@ -1664,7 +1670,7 @@
       </c>
     </row>
     <row r="65" ht="14.25">
-      <c r="A65" s="4">
+      <c r="A65" s="1">
         <v>46100</v>
       </c>
       <c r="B65" t="s">
@@ -1672,6 +1678,17 @@
       </c>
       <c r="C65" s="2" t="s">
         <v>130</v>
+      </c>
+    </row>
+    <row r="66" ht="14.25">
+      <c r="A66" s="4">
+        <v>46101</v>
+      </c>
+      <c r="B66" t="s">
+        <v>131</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1739,6 +1756,7 @@
     <hyperlink r:id="rId61" ref="C63"/>
     <hyperlink r:id="rId62" ref="C64"/>
     <hyperlink r:id="rId63" ref="C65"/>
+    <hyperlink r:id="rId64" ref="C66"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: construction of Binary Trees if either inorder and postorder is given or inorder and preorder is given
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t>date</t>
   </si>
@@ -433,6 +433,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/symmetric-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construct Binary Tree from inorder and preorder traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-preorder-traversal/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Construct Binary Tree from inorder and postorder traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-postorder-traversal/</t>
   </si>
 </sst>
 </file>
@@ -473,7 +485,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -481,6 +493,7 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -981,7 +994,7 @@
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col bestFit="1" min="1" max="1" width="12.30078125"/>
-    <col bestFit="1" min="2" max="2" width="35.98046875"/>
+    <col bestFit="1" min="2" max="2" width="51.40234375"/>
     <col bestFit="1" min="3" max="3" width="96.87109375"/>
     <col bestFit="1" min="4" max="4" width="21.69140625"/>
   </cols>
@@ -1732,7 +1745,7 @@
       </c>
     </row>
     <row r="69" ht="14.25">
-      <c r="A69" s="4">
+      <c r="A69" s="1">
         <v>46102</v>
       </c>
       <c r="B69" t="s">
@@ -1740,6 +1753,28 @@
       </c>
       <c r="C69" s="2" t="s">
         <v>138</v>
+      </c>
+    </row>
+    <row r="70" ht="14.25">
+      <c r="A70" s="4">
+        <v>46103</v>
+      </c>
+      <c r="B70" t="s">
+        <v>139</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="71" ht="14.25">
+      <c r="A71" s="4">
+        <v>46103</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1811,6 +1846,8 @@
     <hyperlink r:id="rId65" ref="C67"/>
     <hyperlink r:id="rId66" ref="C68"/>
     <hyperlink r:id="rId67" ref="C69"/>
+    <hyperlink r:id="rId68" ref="C70"/>
+    <hyperlink r:id="rId69" ref="C71"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Populating Next Right Pointers in each node II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t>date</t>
   </si>
@@ -445,6 +445,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/construct-binary-tree-from-inorder-and-postorder-traversal/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Populating next right pointers in each node II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/populating-next-right-pointers-in-each-node-ii/</t>
   </si>
 </sst>
 </file>
@@ -492,8 +498,8 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1756,7 +1762,7 @@
       </c>
     </row>
     <row r="70" ht="14.25">
-      <c r="A70" s="4">
+      <c r="A70" s="1">
         <v>46103</v>
       </c>
       <c r="B70" t="s">
@@ -1767,14 +1773,25 @@
       </c>
     </row>
     <row r="71" ht="14.25">
-      <c r="A71" s="4">
+      <c r="A71" s="1">
         <v>46103</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="4" t="s">
         <v>141</v>
       </c>
       <c r="C71" s="2" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="72" ht="14.25">
+      <c r="A72" s="5">
+        <v>46104</v>
+      </c>
+      <c r="B72" t="s">
+        <v>143</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
   </sheetData>
@@ -1848,6 +1865,7 @@
     <hyperlink r:id="rId67" ref="C69"/>
     <hyperlink r:id="rId68" ref="C70"/>
     <hyperlink r:id="rId69" ref="C71"/>
+    <hyperlink r:id="rId70" ref="C72"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: path sum & path sum II & sum root to leaf numbers
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="159">
   <si>
     <t>date</t>
   </si>
@@ -475,6 +475,24 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/flatten-binary-tree-to-linked-list/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Path Sum </t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/path-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Path Sum II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/path-sum-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sum Root to Leaf numbers</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/sum-root-to-leaf-numbers/</t>
   </si>
 </sst>
 </file>
@@ -1819,7 +1837,7 @@
       </c>
     </row>
     <row r="73" ht="14.25">
-      <c r="A73" s="5">
+      <c r="A73" s="1">
         <v>46105</v>
       </c>
       <c r="B73" t="s">
@@ -1830,7 +1848,7 @@
       </c>
     </row>
     <row r="74" ht="14.25">
-      <c r="A74" s="5">
+      <c r="A74" s="1">
         <v>46105</v>
       </c>
       <c r="B74" t="s">
@@ -1841,7 +1859,7 @@
       </c>
     </row>
     <row r="75" ht="14.25">
-      <c r="A75" s="5">
+      <c r="A75" s="1">
         <v>46105</v>
       </c>
       <c r="B75" t="s">
@@ -1852,7 +1870,7 @@
       </c>
     </row>
     <row r="76" ht="14.25">
-      <c r="A76" s="5">
+      <c r="A76" s="1">
         <v>46105</v>
       </c>
       <c r="B76" t="s">
@@ -1860,6 +1878,39 @@
       </c>
       <c r="C76" s="2" t="s">
         <v>152</v>
+      </c>
+    </row>
+    <row r="77" ht="14.25">
+      <c r="A77" s="5">
+        <v>46106</v>
+      </c>
+      <c r="B77" t="s">
+        <v>153</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="78" ht="14.25">
+      <c r="A78" s="5">
+        <v>46106</v>
+      </c>
+      <c r="B78" t="s">
+        <v>155</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="79" ht="14.25">
+      <c r="A79" s="5">
+        <v>46106</v>
+      </c>
+      <c r="B79" t="s">
+        <v>157</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>
@@ -1938,6 +1989,9 @@
     <hyperlink r:id="rId72" ref="C74"/>
     <hyperlink r:id="rId73" ref="C75"/>
     <hyperlink r:id="rId74" ref="C76"/>
+    <hyperlink r:id="rId75" ref="C77"/>
+    <hyperlink r:id="rId76" ref="C78"/>
+    <hyperlink r:id="rId77" ref="C79"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Binary Tree Right-side View
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
   <si>
     <t>date</t>
   </si>
@@ -517,6 +517,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary tree right side view</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-right-side-view/</t>
   </si>
 </sst>
 </file>
@@ -1971,7 +1977,7 @@
       </c>
     </row>
     <row r="83" ht="14.25">
-      <c r="A83" s="5">
+      <c r="A83" s="1">
         <v>46108</v>
       </c>
       <c r="B83" t="s">
@@ -1979,6 +1985,17 @@
       </c>
       <c r="C83" s="2" t="s">
         <v>166</v>
+      </c>
+    </row>
+    <row r="84" ht="14.25">
+      <c r="A84" s="5">
+        <v>46108</v>
+      </c>
+      <c r="B84" t="s">
+        <v>167</v>
+      </c>
+      <c r="C84" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -2064,6 +2081,7 @@
     <hyperlink r:id="rId79" ref="C81"/>
     <hyperlink r:id="rId80" ref="C82"/>
     <hyperlink r:id="rId81" ref="C83"/>
+    <hyperlink r:id="rId82" ref="C84"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: Avg of levels in binary tree
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
   <si>
     <t>date</t>
   </si>
@@ -523,6 +523,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/binary-tree-right-side-view/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avg of levels in Binary Tree</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/average-of-levels-in-binary-tree/</t>
   </si>
 </sst>
 </file>
@@ -1988,7 +1994,7 @@
       </c>
     </row>
     <row r="84" ht="14.25">
-      <c r="A84" s="5">
+      <c r="A84" s="1">
         <v>46108</v>
       </c>
       <c r="B84" t="s">
@@ -1996,6 +2002,17 @@
       </c>
       <c r="C84" s="2" t="s">
         <v>168</v>
+      </c>
+    </row>
+    <row r="85" ht="14.25">
+      <c r="A85" s="5">
+        <v>46108</v>
+      </c>
+      <c r="B85" t="s">
+        <v>169</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -2082,6 +2099,7 @@
     <hyperlink r:id="rId80" ref="C82"/>
     <hyperlink r:id="rId81" ref="C83"/>
     <hyperlink r:id="rId82" ref="C84"/>
+    <hyperlink r:id="rId83" ref="C85"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: binary tree levelOrder traversal
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
   <si>
     <t>date</t>
   </si>
@@ -529,6 +529,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/average-of-levels-in-binary-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binary Tree level-order traversal</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/binary-tree-level-order-traversal/</t>
   </si>
 </sst>
 </file>
@@ -2005,7 +2011,7 @@
       </c>
     </row>
     <row r="85" ht="14.25">
-      <c r="A85" s="5">
+      <c r="A85" s="1">
         <v>46108</v>
       </c>
       <c r="B85" t="s">
@@ -2013,6 +2019,17 @@
       </c>
       <c r="C85" s="2" t="s">
         <v>170</v>
+      </c>
+    </row>
+    <row r="86" ht="14.25">
+      <c r="A86" s="5">
+        <v>46109</v>
+      </c>
+      <c r="B86" t="s">
+        <v>171</v>
+      </c>
+      <c r="C86" s="2" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -2100,6 +2117,7 @@
     <hyperlink r:id="rId81" ref="C83"/>
     <hyperlink r:id="rId82" ref="C84"/>
     <hyperlink r:id="rId83" ref="C85"/>
+    <hyperlink r:id="rId84" ref="C86"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problems: no. of set bits, reverse bits
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="199">
   <si>
     <t>date</t>
   </si>
@@ -601,6 +601,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/add-binary/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reverse Bits</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/reverse-bits/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no. of set bits(Hamming Weight)</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/number-of-1-bits/</t>
   </si>
 </sst>
 </file>
@@ -2209,7 +2221,7 @@
       </c>
     </row>
     <row r="97" ht="14.25">
-      <c r="A97" s="5">
+      <c r="A97" s="1">
         <v>46113</v>
       </c>
       <c r="B97" t="s">
@@ -2217,6 +2229,28 @@
       </c>
       <c r="C97" s="2" t="s">
         <v>194</v>
+      </c>
+    </row>
+    <row r="98" ht="14.25">
+      <c r="A98" s="5">
+        <v>46113</v>
+      </c>
+      <c r="B98" t="s">
+        <v>195</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="99" ht="14.25">
+      <c r="A99" s="5">
+        <v>46113</v>
+      </c>
+      <c r="B99" t="s">
+        <v>197</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -2316,6 +2350,8 @@
     <hyperlink r:id="rId93" ref="C95"/>
     <hyperlink r:id="rId94" ref="C96"/>
     <hyperlink r:id="rId95" ref="C97"/>
+    <hyperlink r:id="rId96" ref="C98"/>
+    <hyperlink r:id="rId97" ref="C99"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: kth largest element in an array
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="205">
   <si>
     <t>date</t>
   </si>
@@ -625,6 +625,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/bitwise-and-of-numbers-range/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kth largest element in an array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/kth-largest-element-in-an-array/</t>
   </si>
 </sst>
 </file>
@@ -2277,7 +2283,7 @@
       </c>
     </row>
     <row r="101" ht="14.25">
-      <c r="A101" s="5">
+      <c r="A101" s="1">
         <v>46114</v>
       </c>
       <c r="B101" t="s">
@@ -2285,6 +2291,17 @@
       </c>
       <c r="C101" s="2" t="s">
         <v>202</v>
+      </c>
+    </row>
+    <row r="102" ht="14.25">
+      <c r="A102" s="5">
+        <v>46114</v>
+      </c>
+      <c r="B102" t="s">
+        <v>203</v>
+      </c>
+      <c r="C102" s="2" t="s">
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -2388,6 +2405,7 @@
     <hyperlink r:id="rId97" ref="C99"/>
     <hyperlink r:id="rId98" ref="C100"/>
     <hyperlink r:id="rId99" ref="C101"/>
+    <hyperlink r:id="rId100" ref="C102"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: valid paranthesis and next greater element
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="225">
   <si>
     <t>date</t>
   </si>
@@ -679,6 +679,18 @@
   </si>
   <si>
     <t>https://www.geeksforgeeks.org/problems/prefix-sum-range-query/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valid paranthesis</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/valid-parentheses/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">next greater element</t>
+  </si>
+  <si>
+    <t>https://www.geeksforgeeks.org/problems/next-larger-element-1587115620/1</t>
   </si>
 </sst>
 </file>
@@ -2419,7 +2431,7 @@
       </c>
     </row>
     <row r="109" ht="14.25">
-      <c r="A109" s="5">
+      <c r="A109" s="1">
         <v>46118</v>
       </c>
       <c r="B109" t="s">
@@ -2430,7 +2442,7 @@
       </c>
     </row>
     <row r="110" ht="14.25">
-      <c r="A110" s="5">
+      <c r="A110" s="1">
         <v>46118</v>
       </c>
       <c r="B110" t="s">
@@ -2438,6 +2450,28 @@
       </c>
       <c r="C110" s="2" t="s">
         <v>220</v>
+      </c>
+    </row>
+    <row r="111" ht="14.25">
+      <c r="A111" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B111" t="s">
+        <v>221</v>
+      </c>
+      <c r="C111" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="112" ht="14.25">
+      <c r="A112" s="5">
+        <v>46118</v>
+      </c>
+      <c r="B112" t="s">
+        <v>223</v>
+      </c>
+      <c r="C112" s="2" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>
@@ -2550,6 +2584,8 @@
     <hyperlink r:id="rId106" ref="C108"/>
     <hyperlink r:id="rId107" ref="C109"/>
     <hyperlink r:id="rId108" ref="C110"/>
+    <hyperlink r:id="rId109" ref="C111"/>
+    <hyperlink r:id="rId110" ref="C112"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem : find first and last position of element in sorted array
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="231">
   <si>
     <t>date</t>
   </si>
@@ -703,6 +703,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/search-in-rotated-sorted-array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">find first and last position of element in sorted array</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
   </si>
 </sst>
 </file>
@@ -2498,7 +2504,7 @@
       </c>
     </row>
     <row r="114" ht="14.25">
-      <c r="A114" s="5">
+      <c r="A114" s="1">
         <v>46119</v>
       </c>
       <c r="B114" t="s">
@@ -2506,6 +2512,17 @@
       </c>
       <c r="C114" s="2" t="s">
         <v>228</v>
+      </c>
+    </row>
+    <row r="115" ht="14.25">
+      <c r="A115" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B115" t="s">
+        <v>229</v>
+      </c>
+      <c r="C115" s="2" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -2622,6 +2639,7 @@
     <hyperlink r:id="rId110" ref="C112"/>
     <hyperlink r:id="rId111" ref="C113"/>
     <hyperlink r:id="rId112" ref="C114"/>
+    <hyperlink r:id="rId113" ref="C115"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: convert sorted array to BST
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="247">
   <si>
     <t>date</t>
   </si>
@@ -751,6 +751,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/maximum-sum-circular-subarray/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">convert sorted array to BST</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/convert-sorted-array-to-binary-search-tree/</t>
   </si>
 </sst>
 </file>
@@ -799,10 +805,10 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
       <protection hidden="0" locked="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2637,14 +2643,25 @@
       </c>
     </row>
     <row r="122" ht="14.25">
-      <c r="A122" s="5">
+      <c r="A122" s="1">
         <v>46123</v>
       </c>
       <c r="B122" t="s">
         <v>243</v>
       </c>
-      <c r="C122" s="6" t="s">
+      <c r="C122" s="5" t="s">
         <v>244</v>
+      </c>
+    </row>
+    <row r="123" ht="14.25">
+      <c r="A123" s="6">
+        <v>46123</v>
+      </c>
+      <c r="B123" t="s">
+        <v>245</v>
+      </c>
+      <c r="C123" s="2" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -2769,6 +2786,7 @@
     <hyperlink r:id="rId118" ref="C120"/>
     <hyperlink r:id="rId119" ref="C121"/>
     <hyperlink r:id="rId120" ref="C122"/>
+    <hyperlink r:id="rId121" ref="C123"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: merge k sorted LLs
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="253">
   <si>
     <t>date</t>
   </si>
@@ -769,6 +769,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/construct-quad-tree/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merge k sorted lists</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
   </si>
 </sst>
 </file>
@@ -2688,7 +2694,7 @@
       </c>
     </row>
     <row r="125" ht="14.25">
-      <c r="A125" s="6">
+      <c r="A125" s="1">
         <v>46124</v>
       </c>
       <c r="B125" t="s">
@@ -2696,6 +2702,17 @@
       </c>
       <c r="C125" s="2" t="s">
         <v>250</v>
+      </c>
+    </row>
+    <row r="126" ht="14.25">
+      <c r="A126" s="6">
+        <v>46124</v>
+      </c>
+      <c r="B126" t="s">
+        <v>251</v>
+      </c>
+      <c r="C126" s="2" t="s">
+        <v>252</v>
       </c>
     </row>
   </sheetData>
@@ -2823,6 +2840,7 @@
     <hyperlink r:id="rId121" ref="C123"/>
     <hyperlink r:id="rId122" ref="C124"/>
     <hyperlink r:id="rId123" ref="C125"/>
+    <hyperlink r:id="rId124" ref="C126"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem : design add and search words data structure
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
   <si>
     <t>date</t>
   </si>
@@ -775,6 +775,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/merge-k-sorted-lists/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">design add and search words Data Structures</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/design-add-and-search-words-data-structure/</t>
   </si>
 </sst>
 </file>
@@ -2705,7 +2711,7 @@
       </c>
     </row>
     <row r="126" ht="14.25">
-      <c r="A126" s="6">
+      <c r="A126" s="1">
         <v>46124</v>
       </c>
       <c r="B126" t="s">
@@ -2713,6 +2719,17 @@
       </c>
       <c r="C126" s="2" t="s">
         <v>252</v>
+      </c>
+    </row>
+    <row r="127" ht="14.25">
+      <c r="A127" s="6">
+        <v>46125</v>
+      </c>
+      <c r="B127" t="s">
+        <v>253</v>
+      </c>
+      <c r="C127" s="2" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -2841,6 +2858,7 @@
     <hyperlink r:id="rId122" ref="C124"/>
     <hyperlink r:id="rId123" ref="C125"/>
     <hyperlink r:id="rId124" ref="C126"/>
+    <hyperlink r:id="rId125" ref="C127"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: word search II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="257">
   <si>
     <t>date</t>
   </si>
@@ -781,6 +781,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/design-add-and-search-words-data-structure/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">word search II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/word-search-ii/</t>
   </si>
 </sst>
 </file>
@@ -2722,7 +2728,7 @@
       </c>
     </row>
     <row r="127" ht="14.25">
-      <c r="A127" s="6">
+      <c r="A127" s="1">
         <v>46125</v>
       </c>
       <c r="B127" t="s">
@@ -2730,6 +2736,17 @@
       </c>
       <c r="C127" s="2" t="s">
         <v>254</v>
+      </c>
+    </row>
+    <row r="128" ht="14.25">
+      <c r="A128" s="6">
+        <v>46126</v>
+      </c>
+      <c r="B128" t="s">
+        <v>255</v>
+      </c>
+      <c r="C128" s="5" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -2859,6 +2876,7 @@
     <hyperlink r:id="rId123" ref="C125"/>
     <hyperlink r:id="rId124" ref="C126"/>
     <hyperlink r:id="rId125" ref="C127"/>
+    <hyperlink r:id="rId126" ref="C128"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: copy list with random pointers
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="259">
   <si>
     <t>date</t>
   </si>
@@ -787,6 +787,12 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/word-search-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">copy list with random pointers</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/copy-list-with-random-pointer/</t>
   </si>
 </sst>
 </file>
@@ -2739,7 +2745,7 @@
       </c>
     </row>
     <row r="128" ht="14.25">
-      <c r="A128" s="6">
+      <c r="A128" s="1">
         <v>46126</v>
       </c>
       <c r="B128" t="s">
@@ -2747,6 +2753,17 @@
       </c>
       <c r="C128" s="5" t="s">
         <v>256</v>
+      </c>
+    </row>
+    <row r="129" ht="14.25">
+      <c r="A129" s="6">
+        <v>46130</v>
+      </c>
+      <c r="B129" t="s">
+        <v>257</v>
+      </c>
+      <c r="C129" s="2" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -2877,6 +2894,7 @@
     <hyperlink r:id="rId124" ref="C126"/>
     <hyperlink r:id="rId125" ref="C127"/>
     <hyperlink r:id="rId126" ref="C128"/>
+    <hyperlink r:id="rId127" ref="C129"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: contains duplicate II
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
   <si>
     <t>date</t>
   </si>
@@ -913,12 +913,21 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/happy-number/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">contains duplicate II</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-1070000]d/mm/yyyy;@"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11.000000"/>
@@ -953,9 +962,9 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -964,7 +973,6 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1464,14 +1472,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col bestFit="1" min="1" max="1" width="12.30078125"/>
+    <col bestFit="1" min="1" max="1" style="1" width="12.30078125"/>
     <col bestFit="1" min="2" max="2" width="51.40234375"/>
     <col bestFit="1" min="3" max="3" width="96.87109375"/>
     <col bestFit="1" min="4" max="4" width="21.69140625"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -1639,7 +1647,7 @@
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" t="s">
+      <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
     </row>
@@ -3096,7 +3104,7 @@
       </c>
     </row>
     <row r="149" ht="14.25">
-      <c r="A149" s="6">
+      <c r="A149" s="1">
         <v>46144</v>
       </c>
       <c r="B149" t="s">
@@ -3104,6 +3112,17 @@
       </c>
       <c r="C149" s="2" t="s">
         <v>298</v>
+      </c>
+    </row>
+    <row r="150" ht="14.25">
+      <c r="A150" s="1">
+        <v>46058</v>
+      </c>
+      <c r="B150" t="s">
+        <v>299</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -3255,6 +3274,7 @@
     <hyperlink r:id="rId145" ref="C147"/>
     <hyperlink r:id="rId146" ref="C148"/>
     <hyperlink r:id="rId147" ref="C149"/>
+    <hyperlink r:id="rId148" ref="C150"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Problem: longest consecutive sequence
</commit_message>
<xml_diff>
--- a/TrackingQuestions.xlsx
+++ b/TrackingQuestions.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="301" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="303">
   <si>
     <t>date</t>
   </si>
@@ -919,15 +919,18 @@
   </si>
   <si>
     <t>https://leetcode.com/problems/contains-duplicate-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">longest consecutive sequence</t>
+  </si>
+  <si>
+    <t>https://leetcode.com/problems/longest-consecutive-sequence/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="[$-1070000]d/mm/yyyy;@"/>
-  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11.000000"/>
@@ -964,7 +967,7 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
@@ -3116,13 +3119,24 @@
     </row>
     <row r="150" ht="14.25">
       <c r="A150" s="1">
-        <v>46058</v>
+        <v>46144</v>
       </c>
       <c r="B150" t="s">
         <v>299</v>
       </c>
       <c r="C150" s="2" t="s">
         <v>300</v>
+      </c>
+    </row>
+    <row r="151" ht="14.25">
+      <c r="A151" s="1">
+        <v>46145</v>
+      </c>
+      <c r="B151" t="s">
+        <v>301</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -3275,6 +3289,7 @@
     <hyperlink r:id="rId146" ref="C148"/>
     <hyperlink r:id="rId147" ref="C149"/>
     <hyperlink r:id="rId148" ref="C150"/>
+    <hyperlink r:id="rId149" ref="C151"/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>